<commit_message>
sync recent code updates
</commit_message>
<xml_diff>
--- a/CDE_ID_detective_revamp/KnowledgeBase/Compiled_CORE_CDEs list_English_one sheet_as of 2025-01-28.xlsx
+++ b/CDE_ID_detective_revamp/KnowledgeBase/Compiled_CORE_CDEs list_English_one sheet_as of 2025-01-28.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmaefos\Code Stuffs\CDE_detective\CDE_ID_detective_revamp\KnowledgeBase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F653769-EB35-4B62-AE6D-790CA63A73D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A35DEA1-0990-4A45-BF32-ADBB4480D92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19305" yWindow="6465" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{35A4921A-9D1F-4A50-94BD-2A3998B45EE8}"/>
+    <workbookView xWindow="-38385" yWindow="10680" windowWidth="35760" windowHeight="11265" xr2:uid="{35A4921A-9D1F-4A50-94BD-2A3998B45EE8}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="20" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6997" uniqueCount="1248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7042" uniqueCount="1249">
   <si>
     <t>Study Population Focus</t>
   </si>
@@ -4341,6 +4341,9 @@
   </si>
   <si>
     <t>Patient Health Questionnaire 2 (PHQ2)</t>
+  </si>
+  <si>
+    <t>(blank)</t>
   </si>
 </sst>
 </file>
@@ -4510,7 +4513,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4578,6 +4581,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="6"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -16658,8 +16676,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{06BF0BB1-AF18-42F5-A5F1-83AA7DF4D85D}" name="PivotTable2" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:A38" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{06BF0BB1-AF18-42F5-A5F1-83AA7DF4D85D}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:A83" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="24">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -16673,7 +16691,7 @@
         <item sd="0" m="1" x="29"/>
         <item sd="0" x="4"/>
         <item sd="0" m="1" x="30"/>
-        <item sd="0" x="5"/>
+        <item x="5"/>
         <item sd="0" x="6"/>
         <item sd="0" x="16"/>
         <item sd="0" x="8"/>
@@ -16687,9 +16705,9 @@
         <item sd="0" x="15"/>
         <item sd="0" m="1" x="31"/>
         <item sd="0" x="17"/>
-        <item sd="0" x="18"/>
-        <item sd="0" x="19"/>
-        <item x="20"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item sd="0" x="20"/>
         <item m="1" x="27"/>
         <item sd="0" x="21"/>
         <item sd="0" x="22"/>
@@ -17044,11 +17062,11 @@
         <item sd="0" x="62"/>
         <item sd="0" x="63"/>
         <item sd="0" x="64"/>
-        <item sd="0" x="65"/>
+        <item x="65"/>
         <item sd="0" x="66"/>
-        <item sd="0" x="67"/>
-        <item sd="0" x="68"/>
-        <item sd="0" x="69"/>
+        <item x="67"/>
+        <item x="68"/>
+        <item x="69"/>
         <item sd="0" x="129"/>
         <item sd="0" x="130"/>
         <item sd="0" x="131"/>
@@ -17057,7 +17075,7 @@
         <item sd="0" x="134"/>
         <item sd="0" x="135"/>
         <item sd="0" x="136"/>
-        <item sd="0" x="137"/>
+        <item x="137"/>
         <item sd="0" x="183"/>
         <item sd="0" x="184"/>
         <item t="default" sd="0"/>
@@ -17374,7 +17392,7 @@
     <field x="10"/>
     <field x="11"/>
   </rowFields>
-  <rowItems count="35">
+  <rowItems count="80">
     <i>
       <x v="1"/>
     </i>
@@ -17392,6 +17410,90 @@
     </i>
     <i>
       <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="166"/>
+    </i>
+    <i r="1">
+      <x v="167"/>
+    </i>
+    <i r="1">
+      <x v="168"/>
+    </i>
+    <i r="1">
+      <x v="169"/>
+    </i>
+    <i r="2">
+      <x v="151"/>
+    </i>
+    <i r="3">
+      <x v="172"/>
+    </i>
+    <i r="4">
+      <x v="9"/>
+    </i>
+    <i r="5">
+      <x v="35"/>
+    </i>
+    <i r="6">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="170"/>
+    </i>
+    <i r="1">
+      <x v="171"/>
+    </i>
+    <i r="2">
+      <x v="153"/>
+    </i>
+    <i r="3">
+      <x v="174"/>
+    </i>
+    <i r="4">
+      <x v="9"/>
+    </i>
+    <i r="5">
+      <x v="35"/>
+    </i>
+    <i r="6">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="172"/>
+    </i>
+    <i r="2">
+      <x v="154"/>
+    </i>
+    <i r="3">
+      <x v="175"/>
+    </i>
+    <i r="4">
+      <x v="9"/>
+    </i>
+    <i r="5">
+      <x v="35"/>
+    </i>
+    <i r="6">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="173"/>
+    </i>
+    <i r="2">
+      <x v="155"/>
+    </i>
+    <i r="3">
+      <x v="176"/>
+    </i>
+    <i r="4">
+      <x v="31"/>
+    </i>
+    <i r="5">
+      <x v="34"/>
+    </i>
+    <i r="6">
+      <x v="4"/>
     </i>
     <i>
       <x v="9"/>
@@ -17432,35 +17534,86 @@
     <i>
       <x v="22"/>
     </i>
+    <i r="1">
+      <x v="120"/>
+    </i>
+    <i r="1">
+      <x v="121"/>
+    </i>
+    <i r="1">
+      <x v="174"/>
+    </i>
+    <i r="1">
+      <x v="175"/>
+    </i>
+    <i r="1">
+      <x v="176"/>
+    </i>
+    <i r="1">
+      <x v="177"/>
+    </i>
+    <i r="1">
+      <x v="178"/>
+    </i>
+    <i r="1">
+      <x v="179"/>
+    </i>
+    <i r="1">
+      <x v="180"/>
+    </i>
     <i>
       <x v="23"/>
     </i>
+    <i r="1">
+      <x v="120"/>
+    </i>
+    <i r="1">
+      <x v="121"/>
+    </i>
+    <i r="1">
+      <x v="174"/>
+    </i>
+    <i r="1">
+      <x v="175"/>
+    </i>
+    <i r="1">
+      <x v="176"/>
+    </i>
+    <i r="1">
+      <x v="177"/>
+    </i>
+    <i r="1">
+      <x v="178"/>
+    </i>
+    <i r="1">
+      <x v="179"/>
+    </i>
+    <i r="1">
+      <x v="180"/>
+    </i>
+    <i r="1">
+      <x v="181"/>
+    </i>
+    <i r="1">
+      <x v="182"/>
+    </i>
+    <i r="2">
+      <x v="164"/>
+    </i>
+    <i r="3">
+      <x v="185"/>
+    </i>
+    <i r="4">
+      <x v="21"/>
+    </i>
+    <i r="5">
+      <x v="36"/>
+    </i>
+    <i r="6">
+      <x v="4"/>
+    </i>
     <i>
       <x v="24"/>
-    </i>
-    <i r="1">
-      <x v="123"/>
-    </i>
-    <i r="1">
-      <x v="124"/>
-    </i>
-    <i r="1">
-      <x v="125"/>
-    </i>
-    <i r="1">
-      <x v="126"/>
-    </i>
-    <i r="1">
-      <x v="127"/>
-    </i>
-    <i r="1">
-      <x v="128"/>
-    </i>
-    <i r="1">
-      <x v="129"/>
-    </i>
-    <i r="1">
-      <x v="130"/>
     </i>
     <i>
       <x v="26"/>
@@ -23639,7 +23792,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="100" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A100" s="8" t="s">
         <v>997</v>
       </c>
@@ -23695,7 +23848,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="101" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A101" s="8" t="s">
         <v>997</v>
       </c>
@@ -23751,7 +23904,7 @@
         <v>1221</v>
       </c>
     </row>
-    <row r="102" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A102" s="8" t="s">
         <v>997</v>
       </c>
@@ -23804,7 +23957,7 @@
         <v>1222</v>
       </c>
     </row>
-    <row r="103" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A103" s="8" t="s">
         <v>997</v>
       </c>
@@ -23857,7 +24010,7 @@
         <v>1223</v>
       </c>
     </row>
-    <row r="104" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A104" s="8" t="s">
         <v>997</v>
       </c>
@@ -23910,7 +24063,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="105" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A105" s="8" t="s">
         <v>997</v>
       </c>
@@ -23963,7 +24116,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="106" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A106" s="8" t="s">
         <v>997</v>
       </c>
@@ -24016,7 +24169,7 @@
         <v>1226</v>
       </c>
     </row>
-    <row r="107" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A107" s="8" t="s">
         <v>997</v>
       </c>
@@ -24066,7 +24219,7 @@
         <v>1228</v>
       </c>
     </row>
-    <row r="108" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A108" s="8" t="s">
         <v>320</v>
       </c>
@@ -24122,7 +24275,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="109" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A109" s="8" t="s">
         <v>320</v>
       </c>
@@ -24178,7 +24331,7 @@
         <v>1221</v>
       </c>
     </row>
-    <row r="110" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A110" s="8" t="s">
         <v>320</v>
       </c>
@@ -24231,7 +24384,7 @@
         <v>1222</v>
       </c>
     </row>
-    <row r="111" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A111" s="8" t="s">
         <v>320</v>
       </c>
@@ -24284,7 +24437,7 @@
         <v>1223</v>
       </c>
     </row>
-    <row r="112" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A112" s="8" t="s">
         <v>320</v>
       </c>
@@ -24337,7 +24490,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="113" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A113" s="8" t="s">
         <v>320</v>
       </c>
@@ -24390,7 +24543,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="114" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A114" s="8" t="s">
         <v>320</v>
       </c>
@@ -24443,7 +24596,7 @@
         <v>1226</v>
       </c>
     </row>
-    <row r="115" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A115" s="8" t="s">
         <v>320</v>
       </c>
@@ -24493,7 +24646,7 @@
         <v>1228</v>
       </c>
     </row>
-    <row r="116" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A116" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24549,7 +24702,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="117" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A117" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24605,7 +24758,7 @@
         <v>1221</v>
       </c>
     </row>
-    <row r="118" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A118" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24658,7 +24811,7 @@
         <v>1222</v>
       </c>
     </row>
-    <row r="119" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A119" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24711,7 +24864,7 @@
         <v>1223</v>
       </c>
     </row>
-    <row r="120" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A120" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24764,7 +24917,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="121" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A121" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24817,7 +24970,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="122" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A122" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24870,7 +25023,7 @@
         <v>1226</v>
       </c>
     </row>
-    <row r="123" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A123" s="8" t="s">
         <v>1163</v>
       </c>
@@ -24920,7 +25073,7 @@
         <v>1228</v>
       </c>
     </row>
-    <row r="124" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A124" s="8" t="s">
         <v>1164</v>
       </c>
@@ -24976,7 +25129,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="125" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A125" s="8" t="s">
         <v>1164</v>
       </c>
@@ -25032,7 +25185,7 @@
         <v>1221</v>
       </c>
     </row>
-    <row r="126" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A126" s="8" t="s">
         <v>1164</v>
       </c>
@@ -25085,7 +25238,7 @@
         <v>1222</v>
       </c>
     </row>
-    <row r="127" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A127" s="8" t="s">
         <v>1164</v>
       </c>
@@ -25138,7 +25291,7 @@
         <v>1223</v>
       </c>
     </row>
-    <row r="128" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A128" s="8" t="s">
         <v>1164</v>
       </c>
@@ -25191,7 +25344,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="129" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A129" s="8" t="s">
         <v>1164</v>
       </c>
@@ -25244,7 +25397,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="130" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A130" s="8" t="s">
         <v>1164</v>
       </c>
@@ -25297,7 +25450,7 @@
         <v>1226</v>
       </c>
     </row>
-    <row r="131" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A131" s="8" t="s">
         <v>1164</v>
       </c>
@@ -36128,7 +36281,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="340" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="340" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A340" s="8" t="s">
         <v>997</v>
       </c>
@@ -36178,7 +36331,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="341" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="341" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A341" s="8" t="s">
         <v>997</v>
       </c>
@@ -36228,7 +36381,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="342" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="342" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A342" s="8" t="s">
         <v>997</v>
       </c>
@@ -36278,7 +36431,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="343" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="343" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A343" s="8" t="s">
         <v>997</v>
       </c>
@@ -36328,7 +36481,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="344" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="344" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A344" s="8" t="s">
         <v>997</v>
       </c>
@@ -36378,7 +36531,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="345" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="345" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A345" s="8" t="s">
         <v>997</v>
       </c>
@@ -36428,7 +36581,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="346" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="346" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A346" s="8" t="s">
         <v>997</v>
       </c>
@@ -36475,7 +36628,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="347" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="347" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A347" s="8" t="s">
         <v>997</v>
       </c>
@@ -36519,7 +36672,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="348" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="348" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A348" s="8" t="s">
         <v>320</v>
       </c>
@@ -36569,7 +36722,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="349" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="349" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A349" s="8" t="s">
         <v>320</v>
       </c>
@@ -36619,7 +36772,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="350" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="350" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A350" s="8" t="s">
         <v>320</v>
       </c>
@@ -36669,7 +36822,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="351" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="351" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A351" s="8" t="s">
         <v>320</v>
       </c>
@@ -36719,7 +36872,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="352" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="352" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A352" s="8" t="s">
         <v>320</v>
       </c>
@@ -36769,7 +36922,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="353" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="353" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A353" s="8" t="s">
         <v>320</v>
       </c>
@@ -36819,7 +36972,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="354" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="354" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A354" s="8" t="s">
         <v>320</v>
       </c>
@@ -36866,7 +37019,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="355" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="355" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
       <c r="A355" s="8" t="s">
         <v>320</v>
       </c>
@@ -40962,8 +41115,7 @@
   <autoFilter ref="A1:Y435" xr:uid="{52F8D453-0289-4E16-AB7B-CD7D302713CA}">
     <filterColumn colId="2">
       <filters>
-        <filter val="PROMIS PF Pain"/>
-        <filter val="PROMIS PF Pain 6b"/>
+        <filter val="GAD7"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Y431">
@@ -40987,10 +41139,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B03DD75-91C1-4925-A600-9AD1195ECA81}">
-  <dimension ref="A3:A38"/>
+  <dimension ref="A3:A83"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="35.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="159.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:1" x14ac:dyDescent="0.45">
@@ -41029,147 +41181,372 @@
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A10" s="2" t="s">
-        <v>698</v>
+      <c r="A10" s="23" t="s">
+        <v>1187</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
-        <v>1247</v>
+      <c r="A11" s="23" t="s">
+        <v>1191</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A12" s="2" t="s">
-        <v>1229</v>
+      <c r="A12" s="23" t="s">
+        <v>1195</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
-        <v>499</v>
+      <c r="A13" s="23" t="s">
+        <v>1199</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A14" s="2" t="s">
-        <v>917</v>
+      <c r="A14" s="24" t="s">
+        <v>1198</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A15" s="2" t="s">
-        <v>816</v>
+      <c r="A15" s="25" t="s">
+        <v>1200</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A16" s="2" t="s">
-        <v>697</v>
+      <c r="A16" s="26" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A17" s="2" t="s">
-        <v>469</v>
+      <c r="A17" s="27" t="s">
+        <v>1134</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A18" s="2" t="s">
-        <v>441</v>
+      <c r="A18" s="28" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A19" s="2" t="s">
-        <v>686</v>
+      <c r="A19" s="23" t="s">
+        <v>1203</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A20" s="2" t="s">
-        <v>1016</v>
+      <c r="A20" s="23" t="s">
+        <v>1207</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A21" s="2" t="s">
-        <v>685</v>
+      <c r="A21" s="24" t="s">
+        <v>1206</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A22" s="2" t="s">
-        <v>1111</v>
+      <c r="A22" s="25" t="s">
+        <v>1208</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A23" s="2" t="s">
-        <v>1165</v>
+      <c r="A23" s="26" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A24" s="2" t="s">
-        <v>1001</v>
+      <c r="A24" s="27" t="s">
+        <v>1134</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A25" s="23" t="s">
-        <v>509</v>
+      <c r="A25" s="28" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A26" s="23" t="s">
-        <v>517</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A27" s="23" t="s">
-        <v>513</v>
+      <c r="A27" s="24" t="s">
+        <v>1210</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A28" s="23" t="s">
-        <v>521</v>
+      <c r="A28" s="25" t="s">
+        <v>1212</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A29" s="23" t="s">
-        <v>503</v>
+      <c r="A29" s="26" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A30" s="23" t="s">
-        <v>526</v>
+      <c r="A30" s="27" t="s">
+        <v>1134</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A31" s="23" t="s">
-        <v>530</v>
+      <c r="A31" s="28" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A32" s="23" t="s">
-        <v>533</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A33" s="2" t="s">
-        <v>329</v>
+      <c r="A33" s="24" t="s">
+        <v>1214</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A34" s="2" t="s">
-        <v>322</v>
+      <c r="A34" s="25" t="s">
+        <v>1216</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A35" s="2" t="s">
-        <v>536</v>
+      <c r="A35" s="26" t="s">
+        <v>1248</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A36" s="2" t="s">
-        <v>381</v>
+      <c r="A36" s="27" t="s">
+        <v>1248</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A37" s="2" t="s">
-        <v>1231</v>
+      <c r="A37" s="28" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A39" s="2" t="s">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A40" s="2" t="s">
+        <v>1229</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A41" s="2" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A42" s="2" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A43" s="2" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A44" s="2" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A45" s="2" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A46" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A47" s="2" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A48" s="2" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A49" s="2" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A50" s="2" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A51" s="23" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A52" s="23" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A53" s="23" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A54" s="23" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A55" s="23" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A56" s="23" t="s">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A57" s="23" t="s">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A58" s="23" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A59" s="23" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A60" s="2" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A61" s="23" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A62" s="23" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A63" s="23" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A64" s="23" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A65" s="23" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A66" s="23" t="s">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A67" s="23" t="s">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A68" s="23" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A69" s="23" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A70" s="23" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A71" s="23" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A72" s="24" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A73" s="25" t="s">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A74" s="26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A75" s="27" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A76" s="28" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A77" s="2" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A78" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A79" s="2" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A80" s="2" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A81" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A82" s="2" t="s">
+        <v>1231</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A83" s="2" t="s">
         <v>1021</v>
       </c>
     </row>
@@ -41179,23 +41556,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="3ebfc1ff-6854-40f8-8577-9c1c65c79578" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5B4F2C3D199264E8B8F6DBDBC9FDDAA" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e6ed8d6e314981ace17ace03515ae845">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="3ebfc1ff-6854-40f8-8577-9c1c65c79578" xmlns:ns4="1db1eb16-7f87-45b5-a5c6-bd3f038db8d0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a14e8e53890f120b2bee09526d13603f" ns3:_="" ns4:_="">
     <xsd:import namespace="3ebfc1ff-6854-40f8-8577-9c1c65c79578"/>
@@ -41384,10 +41744,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="3ebfc1ff-6854-40f8-8577-9c1c65c79578" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DFF46F5-41AA-471B-8C04-D49580FCB34E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DDD3AD7-7B2B-4497-B765-450837BD813B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ebfc1ff-6854-40f8-8577-9c1c65c79578"/>
+    <ds:schemaRef ds:uri="1db1eb16-7f87-45b5-a5c6-bd3f038db8d0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -41410,20 +41798,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DDD3AD7-7B2B-4497-B765-450837BD813B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DFF46F5-41AA-471B-8C04-D49580FCB34E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3ebfc1ff-6854-40f8-8577-9c1c65c79578"/>
-    <ds:schemaRef ds:uri="1db1eb16-7f87-45b5-a5c6-bd3f038db8d0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated script to consolidate steps into one file
</commit_message>
<xml_diff>
--- a/CDE_ID_detective_revamp/KnowledgeBase/Compiled_CORE_CDEs list_English_one sheet_as of 2025-01-28.xlsx
+++ b/CDE_ID_detective_revamp/KnowledgeBase/Compiled_CORE_CDEs list_English_one sheet_as of 2025-01-28.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lmaefos\Code Stuffs\CDE_detective\CDE_ID_detective_revamp\KnowledgeBase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A35DEA1-0990-4A45-BF32-ADBB4480D92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89C75B6-9963-4913-8422-2FA1F8AA1453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38385" yWindow="10680" windowWidth="35760" windowHeight="11265" xr2:uid="{35A4921A-9D1F-4A50-94BD-2A3998B45EE8}"/>
+    <workbookView xWindow="-19950" yWindow="6045" windowWidth="18795" windowHeight="15105" xr2:uid="{35A4921A-9D1F-4A50-94BD-2A3998B45EE8}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL" sheetId="1" r:id="rId1"/>
@@ -17966,7 +17966,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F8D453-0289-4E16-AB7B-CD7D302713CA}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:Y435"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -18071,7 +18070,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>997</v>
       </c>
@@ -18085,7 +18084,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="3" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>535</v>
       </c>
@@ -18099,7 +18098,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>1015</v>
       </c>
@@ -18113,7 +18112,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="5" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A5" s="8" t="s">
         <v>535</v>
       </c>
@@ -18166,7 +18165,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="6" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A6" s="8" t="s">
         <v>535</v>
       </c>
@@ -18219,7 +18218,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="7" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A7" s="8" t="s">
         <v>535</v>
       </c>
@@ -18272,7 +18271,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="8" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A8" s="8" t="s">
         <v>535</v>
       </c>
@@ -18325,7 +18324,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="9" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A9" s="8" t="s">
         <v>535</v>
       </c>
@@ -18372,7 +18371,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A10" s="8" t="s">
         <v>997</v>
       </c>
@@ -18425,7 +18424,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="11" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A11" s="8" t="s">
         <v>997</v>
       </c>
@@ -18478,7 +18477,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="12" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A12" s="8" t="s">
         <v>997</v>
       </c>
@@ -18531,7 +18530,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="13" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A13" s="8" t="s">
         <v>997</v>
       </c>
@@ -18584,7 +18583,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="14" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A14" s="8" t="s">
         <v>1015</v>
       </c>
@@ -18637,7 +18636,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="15" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A15" s="8" t="s">
         <v>1015</v>
       </c>
@@ -18690,7 +18689,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="16" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A16" s="8" t="s">
         <v>1015</v>
       </c>
@@ -18743,7 +18742,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="17" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A17" s="8" t="s">
         <v>1015</v>
       </c>
@@ -18796,7 +18795,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="18" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
@@ -18860,7 +18859,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A19" s="8" t="s">
         <v>22</v>
       </c>
@@ -18913,7 +18912,7 @@
       <c r="W19" s="9"/>
       <c r="X19" s="9"/>
     </row>
-    <row r="20" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A20" s="8" t="s">
         <v>22</v>
       </c>
@@ -18976,7 +18975,7 @@
       <c r="W20" s="9"/>
       <c r="X20" s="9"/>
     </row>
-    <row r="21" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A21" s="8" t="s">
         <v>22</v>
       </c>
@@ -19043,7 +19042,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A22" s="8" t="s">
         <v>22</v>
       </c>
@@ -19103,7 +19102,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A23" s="8" t="s">
         <v>22</v>
       </c>
@@ -19166,7 +19165,7 @@
       <c r="W23" s="9"/>
       <c r="X23" s="9"/>
     </row>
-    <row r="24" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A24" s="8" t="s">
         <v>22</v>
       </c>
@@ -19229,7 +19228,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="25" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A25" s="8" t="s">
         <v>22</v>
       </c>
@@ -19292,7 +19291,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="26" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A26" s="8" t="s">
         <v>22</v>
       </c>
@@ -19355,7 +19354,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="27" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A27" s="8" t="s">
         <v>22</v>
       </c>
@@ -19418,7 +19417,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="28" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A28" s="8" t="s">
         <v>22</v>
       </c>
@@ -19481,7 +19480,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="29" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A29" s="8" t="s">
         <v>22</v>
       </c>
@@ -19544,7 +19543,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="30" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A30" s="8" t="s">
         <v>22</v>
       </c>
@@ -19607,7 +19606,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="31" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A31" s="8" t="s">
         <v>22</v>
       </c>
@@ -19674,7 +19673,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="32" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A32" s="8" t="s">
         <v>22</v>
       </c>
@@ -19743,7 +19742,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="33" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A33" s="8" t="s">
         <v>22</v>
       </c>
@@ -19810,7 +19809,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="34" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A34" s="8" t="s">
         <v>22</v>
       </c>
@@ -19868,7 +19867,7 @@
       </c>
       <c r="U34" s="9"/>
     </row>
-    <row r="35" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A35" s="8" t="s">
         <v>22</v>
       </c>
@@ -19922,7 +19921,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="36" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A36" s="8" t="s">
         <v>22</v>
       </c>
@@ -19971,7 +19970,7 @@
       <c r="W36" s="9"/>
       <c r="X36" s="9"/>
     </row>
-    <row r="37" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A37" s="8" t="s">
         <v>22</v>
       </c>
@@ -20028,7 +20027,7 @@
       <c r="W37" s="9"/>
       <c r="X37" s="9"/>
     </row>
-    <row r="38" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A38" s="8" t="s">
         <v>22</v>
       </c>
@@ -20082,7 +20081,7 @@
       <c r="W38" s="9"/>
       <c r="X38" s="9"/>
     </row>
-    <row r="39" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A39" s="8" t="s">
         <v>22</v>
       </c>
@@ -20137,7 +20136,7 @@
       <c r="W39" s="9"/>
       <c r="X39" s="9"/>
     </row>
-    <row r="40" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A40" s="8" t="s">
         <v>202</v>
       </c>
@@ -20205,7 +20204,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A41" s="8" t="s">
         <v>202</v>
       </c>
@@ -20263,7 +20262,7 @@
       <c r="X41" s="9"/>
       <c r="Y41" s="9"/>
     </row>
-    <row r="42" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A42" s="8" t="s">
         <v>202</v>
       </c>
@@ -20321,7 +20320,7 @@
       <c r="X42" s="9"/>
       <c r="Y42" s="9"/>
     </row>
-    <row r="43" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A43" s="8" t="s">
         <v>202</v>
       </c>
@@ -20391,7 +20390,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="44" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A44" s="8" t="s">
         <v>202</v>
       </c>
@@ -20463,7 +20462,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A45" s="8" t="s">
         <v>202</v>
       </c>
@@ -20515,7 +20514,7 @@
       <c r="X45" s="9"/>
       <c r="Y45" s="9"/>
     </row>
-    <row r="46" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A46" s="8" t="s">
         <v>202</v>
       </c>
@@ -20581,7 +20580,7 @@
       <c r="X46" s="9"/>
       <c r="Y46" s="9"/>
     </row>
-    <row r="47" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A47" s="8" t="s">
         <v>202</v>
       </c>
@@ -20647,7 +20646,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="48" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A48" s="8" t="s">
         <v>202</v>
       </c>
@@ -20713,7 +20712,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="49" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A49" s="8" t="s">
         <v>202</v>
       </c>
@@ -20779,7 +20778,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="50" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A50" s="8" t="s">
         <v>202</v>
       </c>
@@ -20845,7 +20844,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="51" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A51" s="8" t="s">
         <v>202</v>
       </c>
@@ -20911,7 +20910,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="52" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A52" s="8" t="s">
         <v>202</v>
       </c>
@@ -20977,7 +20976,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="53" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A53" s="8" t="s">
         <v>202</v>
       </c>
@@ -21043,7 +21042,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="54" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A54" s="8" t="s">
         <v>202</v>
       </c>
@@ -21101,7 +21100,7 @@
       <c r="X54" s="9"/>
       <c r="Y54" s="9"/>
     </row>
-    <row r="55" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A55" s="8" t="s">
         <v>202</v>
       </c>
@@ -21159,7 +21158,7 @@
       <c r="X55" s="9"/>
       <c r="Y55" s="9"/>
     </row>
-    <row r="56" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A56" s="8" t="s">
         <v>202</v>
       </c>
@@ -21223,7 +21222,7 @@
       <c r="X56" s="9"/>
       <c r="Y56" s="9"/>
     </row>
-    <row r="57" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A57" s="8" t="s">
         <v>202</v>
       </c>
@@ -21277,7 +21276,7 @@
       <c r="X57" s="9"/>
       <c r="Y57" s="9"/>
     </row>
-    <row r="58" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A58" s="8" t="s">
         <v>202</v>
       </c>
@@ -21343,7 +21342,7 @@
       <c r="X58" s="9"/>
       <c r="Y58" s="9"/>
     </row>
-    <row r="59" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A59" s="8" t="s">
         <v>202</v>
       </c>
@@ -21409,7 +21408,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="60" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A60" s="8" t="s">
         <v>202</v>
       </c>
@@ -21475,7 +21474,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="61" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A61" s="8" t="s">
         <v>202</v>
       </c>
@@ -21541,7 +21540,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="62" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A62" s="8" t="s">
         <v>202</v>
       </c>
@@ -21607,7 +21606,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="63" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A63" s="8" t="s">
         <v>202</v>
       </c>
@@ -21673,7 +21672,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="64" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A64" s="8" t="s">
         <v>202</v>
       </c>
@@ -21739,7 +21738,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="65" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A65" s="8" t="s">
         <v>202</v>
       </c>
@@ -21805,7 +21804,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="66" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A66" s="8" t="s">
         <v>202</v>
       </c>
@@ -21875,7 +21874,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="67" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A67" s="8" t="s">
         <v>202</v>
       </c>
@@ -21947,7 +21946,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="68" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A68" s="8" t="s">
         <v>202</v>
       </c>
@@ -22017,7 +22016,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="69" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A69" s="8" t="s">
         <v>202</v>
       </c>
@@ -22087,7 +22086,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="70" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A70" s="8" t="s">
         <v>202</v>
       </c>
@@ -22159,7 +22158,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="71" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A71" s="8" t="s">
         <v>202</v>
       </c>
@@ -22225,7 +22224,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="72" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A72" s="8" t="s">
         <v>202</v>
       </c>
@@ -22279,7 +22278,7 @@
       <c r="X72" s="9"/>
       <c r="Y72" s="9"/>
     </row>
-    <row r="73" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A73" s="8" t="s">
         <v>202</v>
       </c>
@@ -22337,7 +22336,7 @@
       <c r="X73" s="9"/>
       <c r="Y73" s="9"/>
     </row>
-    <row r="74" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A74" s="8" t="s">
         <v>202</v>
       </c>
@@ -22393,7 +22392,7 @@
       <c r="X74" s="9"/>
       <c r="Y74" s="9"/>
     </row>
-    <row r="75" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A75" s="8" t="s">
         <v>202</v>
       </c>
@@ -22449,7 +22448,7 @@
       <c r="X75" s="15"/>
       <c r="Y75" s="15"/>
     </row>
-    <row r="76" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A76" s="8" t="s">
         <v>22</v>
       </c>
@@ -22508,7 +22507,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="77" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A77" s="8" t="s">
         <v>22</v>
       </c>
@@ -22567,7 +22566,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="78" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A78" s="8" t="s">
         <v>22</v>
       </c>
@@ -22626,7 +22625,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="79" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A79" s="8" t="s">
         <v>22</v>
       </c>
@@ -22685,7 +22684,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="80" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A80" s="8" t="s">
         <v>22</v>
       </c>
@@ -22744,7 +22743,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="81" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A81" s="8" t="s">
         <v>22</v>
       </c>
@@ -22803,7 +22802,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="82" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A82" s="8" t="s">
         <v>22</v>
       </c>
@@ -22862,7 +22861,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="83" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A83" s="8" t="s">
         <v>22</v>
       </c>
@@ -22921,7 +22920,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="84" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A84" s="8" t="s">
         <v>22</v>
       </c>
@@ -22980,7 +22979,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="85" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A85" s="8" t="s">
         <v>22</v>
       </c>
@@ -23035,7 +23034,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="86" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A86" s="8" t="s">
         <v>22</v>
       </c>
@@ -23090,7 +23089,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="87" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A87" s="8" t="s">
         <v>22</v>
       </c>
@@ -23144,7 +23143,7 @@
       <c r="X87" s="15"/>
       <c r="Y87" s="15"/>
     </row>
-    <row r="88" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A88" s="8" t="s">
         <v>1015</v>
       </c>
@@ -23200,7 +23199,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="89" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A89" s="8" t="s">
         <v>1015</v>
       </c>
@@ -23256,7 +23255,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="90" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A90" s="8" t="s">
         <v>1015</v>
       </c>
@@ -23306,7 +23305,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="91" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A91" s="8" t="s">
         <v>997</v>
       </c>
@@ -23362,7 +23361,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="92" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A92" s="8" t="s">
         <v>997</v>
       </c>
@@ -23418,7 +23417,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="93" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A93" s="8" t="s">
         <v>997</v>
       </c>
@@ -23468,7 +23467,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="94" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A94" s="8" t="s">
         <v>320</v>
       </c>
@@ -23524,7 +23523,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="95" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A95" s="8" t="s">
         <v>320</v>
       </c>
@@ -23580,7 +23579,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="96" spans="1:25" hidden="1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:25" x14ac:dyDescent="0.45">
       <c r="A96" s="8" t="s">
         <v>320</v>
       </c>
@@ -23630,7 +23629,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="97" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A97" s="8" t="s">
         <v>535</v>
       </c>
@@ -23686,7 +23685,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="98" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A98" s="8" t="s">
         <v>535</v>
       </c>
@@ -23742,7 +23741,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="99" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A99" s="8" t="s">
         <v>535</v>
       </c>
@@ -25500,7 +25499,7 @@
         <v>1228</v>
       </c>
     </row>
-    <row r="132" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A132" s="8" t="s">
         <v>535</v>
       </c>
@@ -25550,7 +25549,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="133" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A133" s="8" t="s">
         <v>535</v>
       </c>
@@ -25600,7 +25599,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="134" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A134" s="8" t="s">
         <v>535</v>
       </c>
@@ -25650,7 +25649,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="135" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A135" s="8" t="s">
         <v>535</v>
       </c>
@@ -25700,7 +25699,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="136" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A136" s="8" t="s">
         <v>535</v>
       </c>
@@ -25750,7 +25749,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="137" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A137" s="8" t="s">
         <v>535</v>
       </c>
@@ -25800,7 +25799,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="138" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A138" s="8" t="s">
         <v>535</v>
       </c>
@@ -25850,7 +25849,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="139" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A139" s="8" t="s">
         <v>535</v>
       </c>
@@ -25900,7 +25899,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="140" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A140" s="8" t="s">
         <v>535</v>
       </c>
@@ -25950,7 +25949,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="141" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A141" s="8" t="s">
         <v>535</v>
       </c>
@@ -26000,7 +25999,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="142" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A142" s="8" t="s">
         <v>535</v>
       </c>
@@ -26050,7 +26049,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="143" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A143" s="8" t="s">
         <v>535</v>
       </c>
@@ -26100,7 +26099,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="144" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A144" s="8" t="s">
         <v>535</v>
       </c>
@@ -26150,7 +26149,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="145" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A145" s="8" t="s">
         <v>535</v>
       </c>
@@ -26200,7 +26199,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="146" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A146" s="8" t="s">
         <v>535</v>
       </c>
@@ -26250,7 +26249,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="147" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A147" s="8" t="s">
         <v>535</v>
       </c>
@@ -26300,7 +26299,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="148" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A148" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26350,7 +26349,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="149" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A149" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26400,7 +26399,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="150" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A150" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26450,7 +26449,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="151" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A151" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26500,7 +26499,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="152" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A152" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26550,7 +26549,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="153" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A153" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26600,7 +26599,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="154" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A154" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26650,7 +26649,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="155" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A155" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26700,7 +26699,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="156" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A156" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26750,7 +26749,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="157" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A157" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26800,7 +26799,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="158" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A158" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26850,7 +26849,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="159" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A159" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26900,7 +26899,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="160" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A160" s="8" t="s">
         <v>1015</v>
       </c>
@@ -26950,7 +26949,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="161" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A161" s="8" t="s">
         <v>1015</v>
       </c>
@@ -27000,7 +26999,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="162" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A162" s="8" t="s">
         <v>1015</v>
       </c>
@@ -27050,7 +27049,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="163" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A163" s="8" t="s">
         <v>1015</v>
       </c>
@@ -27100,7 +27099,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="164" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A164" s="8" t="s">
         <v>320</v>
       </c>
@@ -27114,7 +27113,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="165" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A165" s="8" t="s">
         <v>997</v>
       </c>
@@ -27128,7 +27127,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="166" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A166" s="8" t="s">
         <v>320</v>
       </c>
@@ -27142,7 +27141,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="167" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A167" s="8" t="s">
         <v>997</v>
       </c>
@@ -27156,7 +27155,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="168" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A168" s="8" t="s">
         <v>535</v>
       </c>
@@ -27209,7 +27208,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="169" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A169" s="8" t="s">
         <v>535</v>
       </c>
@@ -27262,7 +27261,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="170" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A170" s="8" t="s">
         <v>535</v>
       </c>
@@ -27315,7 +27314,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="171" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A171" s="8" t="s">
         <v>535</v>
       </c>
@@ -27368,7 +27367,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="172" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A172" s="8" t="s">
         <v>535</v>
       </c>
@@ -27421,7 +27420,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="173" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A173" s="8" t="s">
         <v>535</v>
       </c>
@@ -27474,7 +27473,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="174" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A174" s="8" t="s">
         <v>535</v>
       </c>
@@ -27527,7 +27526,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="175" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A175" s="8" t="s">
         <v>535</v>
       </c>
@@ -27580,7 +27579,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="176" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A176" s="8" t="s">
         <v>535</v>
       </c>
@@ -27633,7 +27632,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="177" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A177" s="8" t="s">
         <v>535</v>
       </c>
@@ -27686,7 +27685,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="178" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A178" s="8" t="s">
         <v>535</v>
       </c>
@@ -27739,7 +27738,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="179" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="179" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A179" s="8" t="s">
         <v>535</v>
       </c>
@@ -27792,7 +27791,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="180" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="180" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A180" s="8" t="s">
         <v>535</v>
       </c>
@@ -27845,7 +27844,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="181" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="181" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A181" s="8" t="s">
         <v>535</v>
       </c>
@@ -27895,7 +27894,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="182" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A182" s="8" t="s">
         <v>535</v>
       </c>
@@ -27945,7 +27944,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="183" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A183" s="8" t="s">
         <v>535</v>
       </c>
@@ -27995,7 +27994,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="184" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="184" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A184" s="8" t="s">
         <v>535</v>
       </c>
@@ -28045,7 +28044,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="185" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="185" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A185" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28098,7 +28097,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="186" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="186" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A186" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28151,7 +28150,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="187" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="187" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A187" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28204,7 +28203,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="188" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="188" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A188" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28257,7 +28256,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="189" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A189" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28310,7 +28309,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="190" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="190" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A190" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28363,7 +28362,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="191" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A191" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28416,7 +28415,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="192" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="192" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A192" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28469,7 +28468,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="193" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="193" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A193" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28522,7 +28521,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="194" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A194" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28575,7 +28574,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="195" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A195" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28628,7 +28627,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="196" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="196" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A196" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28681,7 +28680,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="197" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A197" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28734,7 +28733,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="198" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="198" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A198" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28784,7 +28783,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="199" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A199" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28834,7 +28833,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="200" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A200" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28884,7 +28883,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="201" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A201" s="8" t="s">
         <v>1015</v>
       </c>
@@ -28934,7 +28933,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="202" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A202" s="8" t="s">
         <v>535</v>
       </c>
@@ -28987,7 +28986,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="203" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="203" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A203" s="8" t="s">
         <v>535</v>
       </c>
@@ -29040,7 +29039,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="204" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A204" s="8" t="s">
         <v>535</v>
       </c>
@@ -29093,7 +29092,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="205" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A205" s="8" t="s">
         <v>535</v>
       </c>
@@ -29146,7 +29145,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="206" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="206" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A206" s="8" t="s">
         <v>535</v>
       </c>
@@ -29199,7 +29198,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="207" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A207" s="8" t="s">
         <v>535</v>
       </c>
@@ -29252,7 +29251,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="208" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="208" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A208" s="8" t="s">
         <v>535</v>
       </c>
@@ -29305,7 +29304,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="209" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A209" s="8" t="s">
         <v>535</v>
       </c>
@@ -29358,7 +29357,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="210" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A210" s="8" t="s">
         <v>535</v>
       </c>
@@ -29411,7 +29410,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="211" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A211" s="8" t="s">
         <v>535</v>
       </c>
@@ -29464,7 +29463,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="212" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="212" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A212" s="8" t="s">
         <v>535</v>
       </c>
@@ -29517,7 +29516,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="213" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="213" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A213" s="8" t="s">
         <v>535</v>
       </c>
@@ -29570,7 +29569,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="214" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A214" s="8" t="s">
         <v>535</v>
       </c>
@@ -29623,7 +29622,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="215" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A215" s="8" t="s">
         <v>535</v>
       </c>
@@ -29673,7 +29672,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="216" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="216" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A216" s="8" t="s">
         <v>535</v>
       </c>
@@ -29723,7 +29722,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="217" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A217" s="8" t="s">
         <v>535</v>
       </c>
@@ -29773,7 +29772,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="218" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A218" s="8" t="s">
         <v>535</v>
       </c>
@@ -29823,7 +29822,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="219" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A219" s="8" t="s">
         <v>1015</v>
       </c>
@@ -29876,7 +29875,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="220" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A220" s="8" t="s">
         <v>1015</v>
       </c>
@@ -29929,7 +29928,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="221" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="221" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A221" s="8" t="s">
         <v>1015</v>
       </c>
@@ -29982,7 +29981,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="222" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="222" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A222" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30035,7 +30034,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="223" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A223" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30088,7 +30087,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="224" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A224" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30141,7 +30140,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="225" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="225" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A225" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30194,7 +30193,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="226" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="226" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A226" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30247,7 +30246,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="227" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A227" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30300,7 +30299,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="228" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="228" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A228" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30353,7 +30352,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="229" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="229" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A229" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30406,7 +30405,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="230" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="230" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A230" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30459,7 +30458,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="231" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="231" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A231" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30512,7 +30511,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="232" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="232" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A232" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30562,7 +30561,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="233" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="233" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A233" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30612,7 +30611,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="234" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="234" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A234" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30662,7 +30661,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="235" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="235" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A235" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30712,7 +30711,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="236" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="236" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A236" s="8" t="s">
         <v>535</v>
       </c>
@@ -30726,7 +30725,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="237" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="237" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A237" s="8" t="s">
         <v>1015</v>
       </c>
@@ -30740,7 +30739,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="238" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="238" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A238" s="8" t="s">
         <v>320</v>
       </c>
@@ -30790,7 +30789,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="239" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="239" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A239" s="8" t="s">
         <v>320</v>
       </c>
@@ -30843,7 +30842,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="240" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="240" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A240" s="8" t="s">
         <v>320</v>
       </c>
@@ -30896,7 +30895,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="241" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="241" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A241" s="8" t="s">
         <v>320</v>
       </c>
@@ -30943,7 +30942,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="242" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="242" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A242" s="8" t="s">
         <v>320</v>
       </c>
@@ -30996,7 +30995,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="243" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="243" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A243" s="8" t="s">
         <v>535</v>
       </c>
@@ -31049,7 +31048,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="244" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="244" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A244" s="8" t="s">
         <v>997</v>
       </c>
@@ -31102,7 +31101,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="245" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="245" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A245" s="8" t="s">
         <v>1015</v>
       </c>
@@ -31155,7 +31154,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="246" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="246" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A246" s="8" t="s">
         <v>535</v>
       </c>
@@ -31208,7 +31207,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="247" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="247" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A247" s="8" t="s">
         <v>1015</v>
       </c>
@@ -31261,7 +31260,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="248" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="248" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A248" s="8" t="s">
         <v>320</v>
       </c>
@@ -31314,7 +31313,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="249" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="249" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A249" s="8" t="s">
         <v>320</v>
       </c>
@@ -31367,7 +31366,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="250" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="250" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A250" s="8" t="s">
         <v>320</v>
       </c>
@@ -31417,7 +31416,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="251" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="251" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A251" s="8" t="s">
         <v>535</v>
       </c>
@@ -31470,7 +31469,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="252" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="252" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A252" s="8" t="s">
         <v>535</v>
       </c>
@@ -31523,7 +31522,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="253" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="253" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A253" s="8" t="s">
         <v>535</v>
       </c>
@@ -31573,7 +31572,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="254" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="254" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A254" s="8" t="s">
         <v>997</v>
       </c>
@@ -31626,7 +31625,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="255" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="255" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A255" s="8" t="s">
         <v>997</v>
       </c>
@@ -31679,7 +31678,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="256" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="256" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A256" s="8" t="s">
         <v>997</v>
       </c>
@@ -31729,7 +31728,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="257" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="257" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A257" s="8" t="s">
         <v>1015</v>
       </c>
@@ -31782,7 +31781,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="258" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="258" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A258" s="8" t="s">
         <v>1015</v>
       </c>
@@ -31835,7 +31834,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="259" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="259" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A259" s="8" t="s">
         <v>1015</v>
       </c>
@@ -31885,7 +31884,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="260" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="260" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A260" s="8" t="s">
         <v>997</v>
       </c>
@@ -31941,7 +31940,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="261" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="261" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A261" s="8" t="s">
         <v>997</v>
       </c>
@@ -31997,7 +31996,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="262" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="262" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A262" s="8" t="s">
         <v>997</v>
       </c>
@@ -32053,7 +32052,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="263" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="263" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A263" s="8" t="s">
         <v>997</v>
       </c>
@@ -32109,7 +32108,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="264" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="264" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A264" s="8" t="s">
         <v>997</v>
       </c>
@@ -32165,7 +32164,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="265" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="265" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A265" s="8" t="s">
         <v>997</v>
       </c>
@@ -32221,7 +32220,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="266" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="266" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A266" s="8" t="s">
         <v>997</v>
       </c>
@@ -32277,7 +32276,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="267" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="267" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A267" s="8" t="s">
         <v>997</v>
       </c>
@@ -32333,7 +32332,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="268" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="268" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A268" s="8" t="s">
         <v>997</v>
       </c>
@@ -32380,7 +32379,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="269" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="269" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A269" s="8" t="s">
         <v>320</v>
       </c>
@@ -32436,7 +32435,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="270" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="270" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A270" s="8" t="s">
         <v>320</v>
       </c>
@@ -32492,7 +32491,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="271" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="271" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A271" s="8" t="s">
         <v>320</v>
       </c>
@@ -32548,7 +32547,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="272" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="272" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A272" s="8" t="s">
         <v>320</v>
       </c>
@@ -32604,7 +32603,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="273" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="273" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A273" s="8" t="s">
         <v>320</v>
       </c>
@@ -32660,7 +32659,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="274" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="274" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A274" s="8" t="s">
         <v>320</v>
       </c>
@@ -32716,7 +32715,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="275" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="275" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A275" s="8" t="s">
         <v>320</v>
       </c>
@@ -32772,7 +32771,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="276" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="276" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A276" s="8" t="s">
         <v>320</v>
       </c>
@@ -32828,7 +32827,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="277" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="277" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A277" s="8" t="s">
         <v>320</v>
       </c>
@@ -32875,7 +32874,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="278" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="278" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A278" s="8" t="s">
         <v>1163</v>
       </c>
@@ -32931,7 +32930,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="279" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="279" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A279" s="8" t="s">
         <v>1163</v>
       </c>
@@ -32987,7 +32986,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="280" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="280" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A280" s="8" t="s">
         <v>1163</v>
       </c>
@@ -33043,7 +33042,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="281" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="281" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A281" s="8" t="s">
         <v>1163</v>
       </c>
@@ -33099,7 +33098,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="282" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="282" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A282" s="8" t="s">
         <v>1163</v>
       </c>
@@ -33155,7 +33154,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="283" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="283" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A283" s="8" t="s">
         <v>1163</v>
       </c>
@@ -33211,7 +33210,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="284" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="284" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A284" s="8" t="s">
         <v>1163</v>
       </c>
@@ -33267,7 +33266,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="285" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="285" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A285" s="8" t="s">
         <v>1163</v>
       </c>
@@ -33323,7 +33322,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="286" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="286" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A286" s="8" t="s">
         <v>1163</v>
       </c>
@@ -33370,7 +33369,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="287" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="287" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A287" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33426,7 +33425,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="288" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="288" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A288" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33482,7 +33481,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="289" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="289" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A289" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33538,7 +33537,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="290" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="290" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A290" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33594,7 +33593,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="291" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="291" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A291" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33650,7 +33649,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="292" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="292" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A292" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33706,7 +33705,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="293" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="293" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A293" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33762,7 +33761,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="294" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="294" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A294" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33818,7 +33817,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="295" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="295" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A295" s="8" t="s">
         <v>1164</v>
       </c>
@@ -33865,7 +33864,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="296" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="296" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A296" s="8" t="s">
         <v>997</v>
       </c>
@@ -33921,7 +33920,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="297" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="297" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A297" s="8" t="s">
         <v>997</v>
       </c>
@@ -33977,7 +33976,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="298" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="298" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A298" s="8" t="s">
         <v>997</v>
       </c>
@@ -34033,7 +34032,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="299" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="299" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A299" s="8" t="s">
         <v>997</v>
       </c>
@@ -34089,7 +34088,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="300" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="300" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A300" s="8" t="s">
         <v>997</v>
       </c>
@@ -34145,7 +34144,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="301" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="301" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A301" s="8" t="s">
         <v>997</v>
       </c>
@@ -34201,7 +34200,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="302" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="302" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A302" s="8" t="s">
         <v>997</v>
       </c>
@@ -34257,7 +34256,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="303" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="303" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A303" s="8" t="s">
         <v>997</v>
       </c>
@@ -34313,7 +34312,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="304" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="304" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A304" s="8" t="s">
         <v>997</v>
       </c>
@@ -34366,7 +34365,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="305" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="305" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A305" s="8" t="s">
         <v>997</v>
       </c>
@@ -34413,7 +34412,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="306" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="306" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A306" s="8" t="s">
         <v>997</v>
       </c>
@@ -34469,7 +34468,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="307" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="307" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A307" s="8" t="s">
         <v>320</v>
       </c>
@@ -34525,7 +34524,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="308" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="308" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A308" s="8" t="s">
         <v>320</v>
       </c>
@@ -34581,7 +34580,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="309" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="309" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A309" s="8" t="s">
         <v>320</v>
       </c>
@@ -34637,7 +34636,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="310" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="310" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A310" s="8" t="s">
         <v>320</v>
       </c>
@@ -34693,7 +34692,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="311" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="311" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A311" s="8" t="s">
         <v>320</v>
       </c>
@@ -34749,7 +34748,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="312" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="312" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A312" s="8" t="s">
         <v>320</v>
       </c>
@@ -34805,7 +34804,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="313" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="313" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A313" s="8" t="s">
         <v>320</v>
       </c>
@@ -34861,7 +34860,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="314" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="314" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A314" s="8" t="s">
         <v>320</v>
       </c>
@@ -34917,7 +34916,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="315" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="315" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A315" s="8" t="s">
         <v>320</v>
       </c>
@@ -34970,7 +34969,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="316" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="316" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A316" s="8" t="s">
         <v>320</v>
       </c>
@@ -35017,7 +35016,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="317" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="317" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A317" s="8" t="s">
         <v>320</v>
       </c>
@@ -35073,7 +35072,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="318" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="318" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A318" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35129,7 +35128,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="319" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="319" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A319" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35185,7 +35184,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="320" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="320" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A320" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35241,7 +35240,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="321" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="321" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A321" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35297,7 +35296,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="322" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="322" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A322" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35353,7 +35352,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="323" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="323" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A323" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35409,7 +35408,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="324" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="324" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A324" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35465,7 +35464,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="325" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="325" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A325" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35521,7 +35520,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="326" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="326" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A326" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35574,7 +35573,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="327" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="327" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A327" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35621,7 +35620,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="328" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="328" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A328" s="8" t="s">
         <v>1163</v>
       </c>
@@ -35677,7 +35676,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="329" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="329" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A329" s="8" t="s">
         <v>1164</v>
       </c>
@@ -35733,7 +35732,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="330" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="330" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A330" s="8" t="s">
         <v>1164</v>
       </c>
@@ -35789,7 +35788,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="331" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="331" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A331" s="8" t="s">
         <v>1164</v>
       </c>
@@ -35845,7 +35844,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="332" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="332" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A332" s="8" t="s">
         <v>1164</v>
       </c>
@@ -35901,7 +35900,7 @@
         <v>1157</v>
       </c>
     </row>
-    <row r="333" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="333" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A333" s="8" t="s">
         <v>1164</v>
       </c>
@@ -35957,7 +35956,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="334" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="334" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A334" s="8" t="s">
         <v>1164</v>
       </c>
@@ -36013,7 +36012,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="335" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="335" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A335" s="8" t="s">
         <v>1164</v>
       </c>
@@ -36069,7 +36068,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="336" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="336" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A336" s="8" t="s">
         <v>1164</v>
       </c>
@@ -36125,7 +36124,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="337" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="337" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A337" s="8" t="s">
         <v>1164</v>
       </c>
@@ -36178,7 +36177,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="338" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="338" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A338" s="8" t="s">
         <v>1164</v>
       </c>
@@ -36225,7 +36224,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="339" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="339" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A339" s="8" t="s">
         <v>1164</v>
       </c>
@@ -36281,7 +36280,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="340" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="340" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A340" s="8" t="s">
         <v>997</v>
       </c>
@@ -36331,7 +36330,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="341" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="341" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A341" s="8" t="s">
         <v>997</v>
       </c>
@@ -36381,7 +36380,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="342" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="342" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A342" s="8" t="s">
         <v>997</v>
       </c>
@@ -36431,7 +36430,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="343" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="343" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A343" s="8" t="s">
         <v>997</v>
       </c>
@@ -36481,7 +36480,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="344" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="344" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A344" s="8" t="s">
         <v>997</v>
       </c>
@@ -36531,7 +36530,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="345" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="345" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A345" s="8" t="s">
         <v>997</v>
       </c>
@@ -36581,7 +36580,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="346" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="346" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A346" s="8" t="s">
         <v>997</v>
       </c>
@@ -36628,7 +36627,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="347" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="347" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A347" s="8" t="s">
         <v>997</v>
       </c>
@@ -36672,7 +36671,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="348" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="348" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A348" s="8" t="s">
         <v>320</v>
       </c>
@@ -36722,7 +36721,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="349" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="349" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A349" s="8" t="s">
         <v>320</v>
       </c>
@@ -36772,7 +36771,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="350" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="350" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A350" s="8" t="s">
         <v>320</v>
       </c>
@@ -36822,7 +36821,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="351" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="351" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A351" s="8" t="s">
         <v>320</v>
       </c>
@@ -36872,7 +36871,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="352" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="352" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A352" s="8" t="s">
         <v>320</v>
       </c>
@@ -36922,7 +36921,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="353" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="353" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A353" s="8" t="s">
         <v>320</v>
       </c>
@@ -36972,7 +36971,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="354" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="354" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A354" s="8" t="s">
         <v>320</v>
       </c>
@@ -37019,7 +37018,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="355" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="355" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A355" s="8" t="s">
         <v>320</v>
       </c>
@@ -37063,7 +37062,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="356" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="356" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A356" s="8" t="s">
         <v>320</v>
       </c>
@@ -37116,7 +37115,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="357" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="357" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A357" s="8" t="s">
         <v>320</v>
       </c>
@@ -37169,7 +37168,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="358" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="358" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A358" s="8" t="s">
         <v>320</v>
       </c>
@@ -37222,7 +37221,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="359" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="359" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A359" s="8" t="s">
         <v>320</v>
       </c>
@@ -37275,7 +37274,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="360" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="360" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A360" s="8" t="s">
         <v>320</v>
       </c>
@@ -37328,7 +37327,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="361" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="361" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A361" s="8" t="s">
         <v>320</v>
       </c>
@@ -37381,7 +37380,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="362" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="362" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A362" s="8" t="s">
         <v>320</v>
       </c>
@@ -37428,7 +37427,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="363" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="363" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A363" s="8" t="s">
         <v>320</v>
       </c>
@@ -37472,7 +37471,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="364" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="364" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A364" s="8" t="s">
         <v>997</v>
       </c>
@@ -37525,7 +37524,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="365" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="365" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A365" s="8" t="s">
         <v>997</v>
       </c>
@@ -37578,7 +37577,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="366" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="366" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A366" s="8" t="s">
         <v>997</v>
       </c>
@@ -37631,7 +37630,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="367" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="367" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A367" s="8" t="s">
         <v>997</v>
       </c>
@@ -37684,7 +37683,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="368" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="368" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A368" s="8" t="s">
         <v>997</v>
       </c>
@@ -37737,7 +37736,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="369" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="369" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A369" s="8" t="s">
         <v>997</v>
       </c>
@@ -37790,7 +37789,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="370" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="370" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A370" s="8" t="s">
         <v>997</v>
       </c>
@@ -37837,7 +37836,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="371" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="371" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A371" s="8" t="s">
         <v>997</v>
       </c>
@@ -37881,7 +37880,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="372" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="372" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A372" s="8" t="s">
         <v>320</v>
       </c>
@@ -37925,7 +37924,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="373" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="373" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A373" s="8" t="s">
         <v>535</v>
       </c>
@@ -37969,7 +37968,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="374" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="374" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A374" s="8" t="s">
         <v>997</v>
       </c>
@@ -38013,7 +38012,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="375" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="375" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A375" s="8" t="s">
         <v>1015</v>
       </c>
@@ -38057,7 +38056,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="376" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="376" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A376" s="8" t="s">
         <v>535</v>
       </c>
@@ -38110,7 +38109,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="377" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="377" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A377" s="8" t="s">
         <v>535</v>
       </c>
@@ -38160,7 +38159,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="378" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="378" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A378" s="8" t="s">
         <v>535</v>
       </c>
@@ -38210,7 +38209,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="379" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="379" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A379" s="8" t="s">
         <v>535</v>
       </c>
@@ -38263,7 +38262,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="380" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="380" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A380" s="8" t="s">
         <v>535</v>
       </c>
@@ -38313,7 +38312,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="381" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="381" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A381" s="8" t="s">
         <v>535</v>
       </c>
@@ -38366,7 +38365,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="382" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="382" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A382" s="8" t="s">
         <v>535</v>
       </c>
@@ -38416,7 +38415,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="383" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="383" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A383" s="8" t="s">
         <v>535</v>
       </c>
@@ -38466,7 +38465,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="384" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="384" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A384" s="8" t="s">
         <v>535</v>
       </c>
@@ -38519,7 +38518,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="385" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="385" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A385" s="8" t="s">
         <v>535</v>
       </c>
@@ -38569,7 +38568,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="386" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="386" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A386" s="8" t="s">
         <v>535</v>
       </c>
@@ -38622,7 +38621,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="387" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="387" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A387" s="8" t="s">
         <v>535</v>
       </c>
@@ -38672,7 +38671,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="388" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="388" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A388" s="8" t="s">
         <v>535</v>
       </c>
@@ -38725,7 +38724,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="389" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="389" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A389" s="8" t="s">
         <v>535</v>
       </c>
@@ -38775,7 +38774,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="390" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="390" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A390" s="8" t="s">
         <v>535</v>
       </c>
@@ -38828,7 +38827,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="391" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="391" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A391" s="8" t="s">
         <v>535</v>
       </c>
@@ -38878,7 +38877,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="392" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="392" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A392" s="8" t="s">
         <v>535</v>
       </c>
@@ -38931,7 +38930,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="393" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="393" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A393" s="8" t="s">
         <v>535</v>
       </c>
@@ -38981,7 +38980,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="394" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="394" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A394" s="8" t="s">
         <v>535</v>
       </c>
@@ -39031,7 +39030,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="395" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="395" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A395" s="8" t="s">
         <v>535</v>
       </c>
@@ -39081,7 +39080,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="396" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="396" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A396" s="8" t="s">
         <v>535</v>
       </c>
@@ -39131,7 +39130,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="397" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="397" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A397" s="8" t="s">
         <v>535</v>
       </c>
@@ -39181,7 +39180,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="398" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="398" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A398" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39234,7 +39233,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="399" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="399" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A399" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39284,7 +39283,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="400" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="400" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A400" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39334,7 +39333,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="401" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="401" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A401" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39387,7 +39386,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="402" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="402" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A402" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39437,7 +39436,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="403" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="403" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A403" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39490,7 +39489,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="404" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="404" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A404" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39540,7 +39539,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="405" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="405" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A405" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39590,7 +39589,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="406" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="406" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A406" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39643,7 +39642,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="407" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="407" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A407" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39693,7 +39692,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="408" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="408" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A408" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39746,7 +39745,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="409" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="409" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A409" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39796,7 +39795,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="410" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="410" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A410" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39849,7 +39848,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="411" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="411" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A411" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39899,7 +39898,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="412" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="412" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A412" s="8" t="s">
         <v>1015</v>
       </c>
@@ -39952,7 +39951,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="413" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="413" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A413" s="8" t="s">
         <v>1015</v>
       </c>
@@ -40002,7 +40001,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="414" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="414" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A414" s="8" t="s">
         <v>1015</v>
       </c>
@@ -40055,7 +40054,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="415" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="415" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A415" s="8" t="s">
         <v>1015</v>
       </c>
@@ -40105,7 +40104,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="416" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="416" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A416" s="8" t="s">
         <v>1015</v>
       </c>
@@ -40155,7 +40154,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="417" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="417" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A417" s="8" t="s">
         <v>1015</v>
       </c>
@@ -40205,7 +40204,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="418" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="418" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A418" s="8" t="s">
         <v>1015</v>
       </c>
@@ -40255,7 +40254,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="419" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="419" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A419" s="8" t="s">
         <v>1015</v>
       </c>
@@ -40305,7 +40304,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="420" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="420" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A420" s="8" t="s">
         <v>320</v>
       </c>
@@ -40355,7 +40354,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="421" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="421" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A421" s="8" t="s">
         <v>320</v>
       </c>
@@ -40405,7 +40404,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="422" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="422" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A422" s="8" t="s">
         <v>320</v>
       </c>
@@ -40455,7 +40454,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="423" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="423" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A423" s="8" t="s">
         <v>320</v>
       </c>
@@ -40505,7 +40504,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="424" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="424" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A424" s="8" t="s">
         <v>320</v>
       </c>
@@ -40555,7 +40554,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="425" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="425" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A425" s="8" t="s">
         <v>320</v>
       </c>
@@ -40608,7 +40607,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="426" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="426" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A426" s="8" t="s">
         <v>997</v>
       </c>
@@ -40658,7 +40657,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="427" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="427" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A427" s="8" t="s">
         <v>997</v>
       </c>
@@ -40708,7 +40707,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="428" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="428" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A428" s="8" t="s">
         <v>997</v>
       </c>
@@ -40758,7 +40757,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="429" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="429" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A429" s="8" t="s">
         <v>997</v>
       </c>
@@ -40808,7 +40807,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="430" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="430" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A430" s="8" t="s">
         <v>997</v>
       </c>
@@ -40858,7 +40857,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="431" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="431" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A431" s="8" t="s">
         <v>997</v>
       </c>
@@ -40911,7 +40910,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="432" spans="1:24" hidden="1" x14ac:dyDescent="0.45">
+    <row r="432" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A432" s="8" t="s">
         <v>997</v>
       </c>
@@ -40961,7 +40960,7 @@
         <v>1146</v>
       </c>
     </row>
-    <row r="433" spans="1:16" hidden="1" x14ac:dyDescent="0.45">
+    <row r="433" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A433" s="8" t="s">
         <v>997</v>
       </c>
@@ -41011,7 +41010,7 @@
         <v>1146</v>
       </c>
     </row>
-    <row r="434" spans="1:16" hidden="1" x14ac:dyDescent="0.45">
+    <row r="434" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A434" s="8" t="s">
         <v>320</v>
       </c>
@@ -41061,7 +41060,7 @@
         <v>1146</v>
       </c>
     </row>
-    <row r="435" spans="1:16" hidden="1" x14ac:dyDescent="0.45">
+    <row r="435" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A435" s="8" t="s">
         <v>320</v>
       </c>
@@ -41113,11 +41112,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:Y435" xr:uid="{52F8D453-0289-4E16-AB7B-CD7D302713CA}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="GAD7"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Y431">
       <sortCondition ref="C2:C431"/>
     </sortState>
@@ -41745,20 +41739,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="3ebfc1ff-6854-40f8-8577-9c1c65c79578" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="3ebfc1ff-6854-40f8-8577-9c1c65c79578" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -41781,6 +41775,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DFF46F5-41AA-471B-8C04-D49580FCB34E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DFAF0B-A9BC-422F-A722-23A769C31190}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -41795,12 +41797,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DFF46F5-41AA-471B-8C04-D49580FCB34E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>